<commit_message>
Refactor workspace services to replace RoleGroup with Team
- Removed WorkspaceRoleGroupService as it is no longer needed.
- Updated WorkspaceRosterService to use Team instead of RoleGroup for roster assignments and shift definitions.
- Modified WorkspaceShiftDefinitionService to handle shifts based on Team instead of RoleGroup.
- Adjusted WorkspaceStaffService to reference Team instead of RoleGroup in staff-related operations.
- Refined WorkspaceTeamService to eliminate RoleGroup references and streamline team management.
- Revised WorkspaceValidationService to validate against Team instead of RoleGroup.
- Updated database schema to remove RoleGroup references from relevant tables and added Team relationships.
- Adjusted tests across services to reflect changes from RoleGroup to Team, ensuring proper functionality.
</commit_message>
<xml_diff>
--- a/src/main/resources/roster.xlsx
+++ b/src/main/resources/roster.xlsx
@@ -437,7 +437,7 @@
   <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
@@ -450,7 +450,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>role_group</t>
+          <t>team</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -492,7 +492,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>L1_China</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -530,7 +530,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>L1_China</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -568,7 +568,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>L1_China</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -606,7 +606,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>AP_L2</t>
+          <t>AP L2</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -644,7 +644,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>AP_L2</t>
+          <t>AP L2</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>AP_L2</t>
+          <t>AP L2</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -720,7 +720,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>AP_L2</t>
+          <t>AP L2</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -758,7 +758,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>AP_L2</t>
+          <t>AP L2</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -809,7 +809,7 @@
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="9" customWidth="1" min="5" max="5"/>
     <col width="7" customWidth="1" min="6" max="6"/>
@@ -859,7 +859,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>role_group</t>
+          <t>team</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -1046,7 +1046,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>L1_China</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -1221,7 +1221,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>AP_L2</t>
+          <t>AP L2</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -1396,7 +1396,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>AP_L2</t>
+          <t>AP L2</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">

</xml_diff>